<commit_message>
check about 2020 birth data file what are the missong records at least one
</commit_message>
<xml_diff>
--- a/notebooks/2020_Birth/First Stage 2020/01_missing_values.xlsx
+++ b/notebooks/2020_Birth/First Stage 2020/01_missing_values.xlsx
@@ -531,14 +531,14 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Birth_Order</t>
+          <t>Birth_Order2.0</t>
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>26007</v>
+        <v>27218</v>
       </c>
       <c r="C3" s="3" t="n">
-        <v>8.6</v>
+        <v>9</v>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
@@ -546,53 +546,53 @@
         </is>
       </c>
       <c r="E3" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>275705</v>
+        <v>274494</v>
       </c>
       <c r="G3" s="3" t="n">
-        <v>91.40000000000001</v>
+        <v>91</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Birth_Order - Copy</t>
+          <t>Birth_Order</t>
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>26007</v>
+        <v>27218</v>
       </c>
       <c r="C4" s="3" t="n">
-        <v>8.6</v>
+        <v>9</v>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>float64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E4" s="3" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>275705</v>
+        <v>274494</v>
       </c>
       <c r="G4" s="3" t="n">
-        <v>91.40000000000001</v>
+        <v>91</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>Multiple_Birth_Status</t>
+          <t>Race_of_Father</t>
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>4163</v>
+        <v>1231</v>
       </c>
       <c r="C5" s="3" t="n">
-        <v>1.4</v>
+        <v>0.4</v>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
@@ -600,26 +600,26 @@
         </is>
       </c>
       <c r="E5" s="3" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>297549</v>
+        <v>300481</v>
       </c>
       <c r="G5" s="3" t="n">
-        <v>98.59999999999999</v>
+        <v>99.59999999999999</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>Race_of_Father</t>
+          <t>Race_of_Mother</t>
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1231</v>
+        <v>520</v>
       </c>
       <c r="C6" s="3" t="n">
-        <v>0.4</v>
+        <v>0.2</v>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
@@ -630,23 +630,23 @@
         <v>6</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>300481</v>
+        <v>301192</v>
       </c>
       <c r="G6" s="3" t="n">
-        <v>99.59999999999999</v>
+        <v>99.8</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Race_of_Mother</t>
+          <t>Marital_Status</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>520</v>
+        <v>17</v>
       </c>
       <c r="C7" s="3" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
@@ -654,23 +654,23 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>301192</v>
+        <v>301695</v>
       </c>
       <c r="G7" s="3" t="n">
-        <v>99.8</v>
+        <v>100</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Marital_Status</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>17</v>
+        <v>2</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>0</v>
@@ -684,7 +684,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>301695</v>
+        <v>301710</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>100</v>
@@ -693,25 +693,25 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>Registered_Year</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>301710</v>
+        <v>301712</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>100</v>
@@ -720,7 +720,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Registered_Month2.0</t>
+          <t>Registered_Month</t>
         </is>
       </c>
       <c r="B10" s="3" t="n">
@@ -747,7 +747,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Registered_Year</t>
+          <t>Registered_District</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -758,11 +758,11 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>1</v>
+        <v>25</v>
       </c>
       <c r="F11" s="3" t="n">
         <v>301712</v>
@@ -774,7 +774,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Hospital or Not</t>
+          <t>Multiple_Birth_Status</t>
         </is>
       </c>
       <c r="B12" s="3" t="n">
@@ -789,7 +789,7 @@
         </is>
       </c>
       <c r="E12" s="3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F12" s="3" t="n">
         <v>301712</v>
@@ -801,7 +801,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Birth_Month</t>
+          <t>Hospital or Not</t>
         </is>
       </c>
       <c r="B13" s="3" t="n">
@@ -816,7 +816,7 @@
         </is>
       </c>
       <c r="E13" s="3" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="F13" s="3" t="n">
         <v>301712</v>
@@ -828,7 +828,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Birh_Year</t>
+          <t>Birth_Month</t>
         </is>
       </c>
       <c r="B14" s="3" t="n">
@@ -839,11 +839,11 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E14" s="3" t="n">
-        <v>63</v>
+        <v>12</v>
       </c>
       <c r="F14" s="3" t="n">
         <v>301712</v>
@@ -882,7 +882,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Registered_District</t>
+          <t>Birh_Year</t>
         </is>
       </c>
       <c r="B16" s="3" t="n">
@@ -893,11 +893,11 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E16" s="3" t="n">
-        <v>25</v>
+        <v>63</v>
       </c>
       <c r="F16" s="3" t="n">
         <v>301712</v>
@@ -909,7 +909,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Registered_Month</t>
+          <t>Birh_Year 2.0</t>
         </is>
       </c>
       <c r="B17" s="3" t="n">
@@ -920,11 +920,11 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E17" s="3" t="n">
-        <v>12</v>
+        <v>63</v>
       </c>
       <c r="F17" s="3" t="n">
         <v>301712</v>
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="5">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>91489</v>
+        <v>89748</v>
       </c>
     </row>
     <row r="6">
@@ -1064,7 +1064,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>1.68</v>
+        <v>1.65</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
creating complete data files 2020
</commit_message>
<xml_diff>
--- a/notebooks/2020_Birth/First Stage 2020/01_missing_values.xlsx
+++ b/notebooks/2020_Birth/First Stage 2020/01_missing_values.xlsx
@@ -508,7 +508,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>33542</v>
+        <v>33541</v>
       </c>
       <c r="C2" s="3" t="n">
         <v>11.1</v>
@@ -522,7 +522,7 @@
         <v>1853</v>
       </c>
       <c r="F2" s="3" t="n">
-        <v>268170</v>
+        <v>268150</v>
       </c>
       <c r="G2" s="3" t="n">
         <v>88.90000000000001</v>
@@ -535,7 +535,7 @@
         </is>
       </c>
       <c r="B3" s="3" t="n">
-        <v>27218</v>
+        <v>27213</v>
       </c>
       <c r="C3" s="3" t="n">
         <v>9</v>
@@ -549,7 +549,7 @@
         <v>9</v>
       </c>
       <c r="F3" s="3" t="n">
-        <v>274494</v>
+        <v>274478</v>
       </c>
       <c r="G3" s="3" t="n">
         <v>91</v>
@@ -562,7 +562,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>27218</v>
+        <v>27213</v>
       </c>
       <c r="C4" s="3" t="n">
         <v>9</v>
@@ -576,7 +576,7 @@
         <v>9</v>
       </c>
       <c r="F4" s="3" t="n">
-        <v>274494</v>
+        <v>274478</v>
       </c>
       <c r="G4" s="3" t="n">
         <v>91</v>
@@ -589,7 +589,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>1231</v>
+        <v>1219</v>
       </c>
       <c r="C5" s="3" t="n">
         <v>0.4</v>
@@ -603,7 +603,7 @@
         <v>6</v>
       </c>
       <c r="F5" s="3" t="n">
-        <v>300481</v>
+        <v>300472</v>
       </c>
       <c r="G5" s="3" t="n">
         <v>99.59999999999999</v>
@@ -616,7 +616,7 @@
         </is>
       </c>
       <c r="B6" s="3" t="n">
-        <v>520</v>
+        <v>505</v>
       </c>
       <c r="C6" s="3" t="n">
         <v>0.2</v>
@@ -630,7 +630,7 @@
         <v>6</v>
       </c>
       <c r="F6" s="3" t="n">
-        <v>301192</v>
+        <v>301186</v>
       </c>
       <c r="G6" s="3" t="n">
         <v>99.8</v>
@@ -639,11 +639,11 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Marital_Status</t>
+          <t>District_of_Mother</t>
         </is>
       </c>
       <c r="B7" s="3" t="n">
-        <v>17</v>
+        <v>29</v>
       </c>
       <c r="C7" s="3" t="n">
         <v>0</v>
@@ -654,10 +654,10 @@
         </is>
       </c>
       <c r="E7" s="3" t="n">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="F7" s="3" t="n">
-        <v>301695</v>
+        <v>301662</v>
       </c>
       <c r="G7" s="3" t="n">
         <v>100</v>
@@ -666,11 +666,11 @@
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
         <is>
-          <t>Gender</t>
+          <t>Marital_Status</t>
         </is>
       </c>
       <c r="B8" s="3" t="n">
-        <v>2</v>
+        <v>17</v>
       </c>
       <c r="C8" s="3" t="n">
         <v>0</v>
@@ -684,7 +684,7 @@
         <v>2</v>
       </c>
       <c r="F8" s="3" t="n">
-        <v>301710</v>
+        <v>301674</v>
       </c>
       <c r="G8" s="3" t="n">
         <v>100</v>
@@ -693,25 +693,25 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Registered_Year</t>
+          <t>Gender</t>
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="C9" s="3" t="n">
         <v>0</v>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E9" s="3" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F9" s="3" t="n">
-        <v>301712</v>
+        <v>301689</v>
       </c>
       <c r="G9" s="3" t="n">
         <v>100</v>
@@ -738,7 +738,7 @@
         <v>12</v>
       </c>
       <c r="F10" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
       <c r="G10" s="3" t="n">
         <v>100</v>
@@ -747,7 +747,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Registered_District</t>
+          <t>Registered_Year</t>
         </is>
       </c>
       <c r="B11" s="3" t="n">
@@ -758,14 +758,14 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E11" s="3" t="n">
-        <v>25</v>
+        <v>1</v>
       </c>
       <c r="F11" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
       <c r="G11" s="3" t="n">
         <v>100</v>
@@ -792,7 +792,7 @@
         <v>5</v>
       </c>
       <c r="F12" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
       <c r="G12" s="3" t="n">
         <v>100</v>
@@ -819,7 +819,7 @@
         <v>2</v>
       </c>
       <c r="F13" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
       <c r="G13" s="3" t="n">
         <v>100</v>
@@ -846,7 +846,7 @@
         <v>12</v>
       </c>
       <c r="F14" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
       <c r="G14" s="3" t="n">
         <v>100</v>
@@ -873,7 +873,7 @@
         <v>12</v>
       </c>
       <c r="F15" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
       <c r="G15" s="3" t="n">
         <v>100</v>
@@ -900,7 +900,7 @@
         <v>63</v>
       </c>
       <c r="F16" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
       <c r="G16" s="3" t="n">
         <v>100</v>
@@ -927,7 +927,7 @@
         <v>63</v>
       </c>
       <c r="F17" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
       <c r="G17" s="3" t="n">
         <v>100</v>
@@ -936,7 +936,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>Age of Mother</t>
+          <t>Registered_District</t>
         </is>
       </c>
       <c r="B18" s="3" t="n">
@@ -947,14 +947,14 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>int64</t>
+          <t>str</t>
         </is>
       </c>
       <c r="E18" s="3" t="n">
-        <v>47</v>
+        <v>25</v>
       </c>
       <c r="F18" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
       <c r="G18" s="3" t="n">
         <v>100</v>
@@ -963,7 +963,7 @@
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
         <is>
-          <t>District_of_Mother</t>
+          <t>Age of Mother</t>
         </is>
       </c>
       <c r="B19" s="3" t="n">
@@ -974,14 +974,14 @@
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>str</t>
+          <t>int64</t>
         </is>
       </c>
       <c r="E19" s="3" t="n">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="F19" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
       <c r="G19" s="3" t="n">
         <v>100</v>
@@ -1024,7 +1024,7 @@
         </is>
       </c>
       <c r="B2" s="3" t="n">
-        <v>301712</v>
+        <v>301691</v>
       </c>
     </row>
     <row r="3">
@@ -1044,7 +1044,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="5">
@@ -1054,7 +1054,7 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>89748</v>
+        <v>89739</v>
       </c>
     </row>
     <row r="6">

</xml_diff>